<commit_message>
docs: expand AgentHub core code guide
</commit_message>
<xml_diff>
--- a/docs/plans/AgentHub_第一周日计划.xlsx
+++ b/docs/plans/AgentHub_第一周日计划.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="15340" activeTab="2"/>
+    <workbookView windowHeight="15100" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="使用说明" sheetId="1" r:id="rId1"/>
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">使用说明!$A$1:$B$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">核心代码入口!$A$1:$D$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">第一周日计划!$A$1:$K$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">第一周日计划!$A$1:$L$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">每日记录模板!$A$1:$I$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">AI使用边界!$A$1:$B$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">第二周候选方向!$A$1:$G$5</definedName>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="173">
   <si>
     <t>项目</t>
   </si>
@@ -198,6 +198,9 @@
     <t>日期</t>
   </si>
   <si>
+    <t>实际日期</t>
+  </si>
+  <si>
     <t>星期</t>
   </si>
   <si>
@@ -226,9 +229,6 @@
   </si>
   <si>
     <t>备注</t>
-  </si>
-  <si>
-    <t>2026-06-15</t>
   </si>
   <si>
     <t>周一</t>
@@ -446,6 +446,9 @@
   </si>
   <si>
     <t>明天优先做</t>
+  </si>
+  <si>
+    <t>2026-06-15</t>
   </si>
   <si>
     <t>类型</t>
@@ -575,7 +578,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="21">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -594,13 +597,6 @@
     <font>
       <sz val="12"/>
       <color theme="10"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -742,7 +738,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="34">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -752,6 +748,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF305496"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1066,150 +1068,150 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1219,6 +1221,19 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="14" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="6" applyBorder="1" applyAlignment="1">
@@ -1637,7 +1652,7 @@
       <c r="A8" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="10" t="s">
         <v>15</v>
       </c>
     </row>
@@ -1683,7 +1698,7 @@
       <c r="A2" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="9" t="s">
         <v>21</v>
       </c>
       <c r="C2" s="3" t="s">
@@ -1697,7 +1712,7 @@
       <c r="A3" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="9" t="s">
         <v>25</v>
       </c>
       <c r="C3" s="3" t="s">
@@ -1711,7 +1726,7 @@
       <c r="A4" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="9" t="s">
         <v>28</v>
       </c>
       <c r="C4" s="3" t="s">
@@ -1725,7 +1740,7 @@
       <c r="A5" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="9" t="s">
         <v>31</v>
       </c>
       <c r="C5" s="3" t="s">
@@ -1739,7 +1754,7 @@
       <c r="A6" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="9" t="s">
         <v>35</v>
       </c>
       <c r="C6" s="3" t="s">
@@ -1753,7 +1768,7 @@
       <c r="A7" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="9" t="s">
         <v>38</v>
       </c>
       <c r="C7" s="3" t="s">
@@ -1767,7 +1782,7 @@
       <c r="A8" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="9" t="s">
         <v>42</v>
       </c>
       <c r="C8" s="3" t="s">
@@ -1781,7 +1796,7 @@
       <c r="A9" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="9" t="s">
         <v>45</v>
       </c>
       <c r="C9" s="3" t="s">
@@ -1795,7 +1810,7 @@
       <c r="A10" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="9" t="s">
         <v>48</v>
       </c>
       <c r="C10" s="3" t="s">
@@ -1828,22 +1843,23 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelRow="7"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="10" customWidth="1"/>
-    <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="48" customWidth="1"/>
-    <col min="6" max="7" width="42" customWidth="1"/>
-    <col min="8" max="8" width="44" customWidth="1"/>
-    <col min="9" max="9" width="30" customWidth="1"/>
-    <col min="10" max="10" width="12" customWidth="1"/>
-    <col min="11" max="11" width="97.5865384615385" customWidth="1"/>
+    <col min="2" max="2" width="13.6153846153846" customWidth="1"/>
+    <col min="3" max="3" width="5.19230769230769" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="9.42307692307692" customWidth="1"/>
+    <col min="6" max="6" width="48" customWidth="1"/>
+    <col min="7" max="8" width="42" customWidth="1"/>
+    <col min="9" max="9" width="44" customWidth="1"/>
+    <col min="10" max="10" width="30" customWidth="1"/>
+    <col min="11" max="11" width="12" customWidth="1"/>
+    <col min="12" max="12" width="97.5865384615385" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:11">
+    <row r="1" ht="28" customHeight="1" spans="1:12">
       <c r="A1" s="1" t="s">
         <v>51</v>
       </c>
@@ -1877,258 +1893,274 @@
       <c r="K1" s="1" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="2" ht="265" customHeight="1" spans="1:11">
-      <c r="A2" s="2" t="s">
+      <c r="L1" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="B2" s="2" t="s">
+    </row>
+    <row r="2" s="4" customFormat="1" ht="236" spans="1:12">
+      <c r="A2" s="5">
+        <v>46188</v>
+      </c>
+      <c r="B2" s="5">
+        <v>46188</v>
+      </c>
+      <c r="C2" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="D2" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="F2" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="G2" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="H2" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="I2" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="J2" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="K2" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="K2" s="3" t="s">
+      <c r="L2" s="7" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="3" ht="58" customHeight="1" spans="1:11">
+    <row r="3" ht="58" customHeight="1" spans="1:12">
       <c r="A3" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="F3" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="G3" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="H3" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="I3" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="J3" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="K3" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="K3" s="3" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="4" ht="58" customHeight="1" spans="1:11">
+      <c r="L3" s="3" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="4" ht="73" customHeight="1" spans="1:12">
       <c r="A4" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="8">
+        <v>46196</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="D4" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="E4" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="F4" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="G4" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="H4" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="I4" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="J4" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="J4" s="2" t="s">
+      <c r="K4" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="K4" s="3" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="5" ht="58" customHeight="1" spans="1:11">
+      <c r="L4" s="3" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="5" ht="58" customHeight="1" spans="1:12">
       <c r="A5" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="2"/>
+      <c r="C5" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="D5" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="E5" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="F5" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="G5" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="H5" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="H5" s="3" t="s">
+      <c r="I5" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="I5" s="3" t="s">
+      <c r="J5" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="J5" s="2" t="s">
+      <c r="K5" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="K5" s="3" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="6" ht="58" customHeight="1" spans="1:11">
+      <c r="L5" s="3" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="6" ht="58" customHeight="1" spans="1:12">
       <c r="A6" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="2"/>
+      <c r="C6" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="D6" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="E6" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="F6" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="G6" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="G6" s="3" t="s">
+      <c r="H6" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="H6" s="3" t="s">
+      <c r="I6" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="I6" s="3" t="s">
+      <c r="J6" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="J6" s="2" t="s">
+      <c r="K6" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="K6" s="3" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="7" ht="58" customHeight="1" spans="1:11">
+      <c r="L6" s="3" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="7" ht="58" customHeight="1" spans="1:12">
       <c r="A7" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="2"/>
+      <c r="C7" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="D7" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="E7" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="F7" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="G7" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="G7" s="3" t="s">
+      <c r="H7" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="H7" s="3" t="s">
+      <c r="I7" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="I7" s="3" t="s">
+      <c r="J7" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="J7" s="2" t="s">
+      <c r="K7" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="K7" s="3" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="8" ht="58" customHeight="1" spans="1:11">
+      <c r="L7" s="3" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="8" ht="58" customHeight="1" spans="1:12">
       <c r="A8" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="2"/>
+      <c r="C8" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="D8" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="E8" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="F8" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="F8" s="3" t="s">
+      <c r="G8" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="G8" s="3" t="s">
+      <c r="H8" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="H8" s="3" t="s">
+      <c r="I8" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="I8" s="3" t="s">
+      <c r="J8" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="J8" s="2" t="s">
+      <c r="K8" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="K8" s="3" t="s">
+      <c r="L8" s="3" t="s">
         <v>82</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:K8" etc:filterBottomFollowUsedRange="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:L8" etc:filterBottomFollowUsedRange="0">
     <extLst/>
   </autoFilter>
   <dataValidations count="1">
-    <dataValidation type="list" sqref="J2:J8">
+    <dataValidation type="list" sqref="K2:K8">
       <formula1>"未开始,进行中,已完成,阻塞"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2183,7 +2215,7 @@
     </row>
     <row r="2" ht="68" customHeight="1" spans="1:9">
       <c r="A2" s="2" t="s">
-        <v>62</v>
+        <v>133</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>82</v>
@@ -2405,26 +2437,26 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2" ht="68" customHeight="1" spans="1:2">
       <c r="A2" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="3" ht="68" customHeight="1" spans="1:2">
       <c r="A3" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
   </sheetData>
@@ -2452,117 +2484,117 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="2" ht="68" customHeight="1" spans="1:7">
       <c r="A2" s="2" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="3" ht="68" customHeight="1" spans="1:7">
       <c r="A3" s="2" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="4" ht="68" customHeight="1" spans="1:7">
       <c r="A4" s="2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="5" ht="68" customHeight="1" spans="1:7">
       <c r="A5" s="2" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
   </sheetData>

</xml_diff>